<commit_message>
fixed the bug in the resignning part
</commit_message>
<xml_diff>
--- a/tickets.xlsx
+++ b/tickets.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +466,11 @@
           <t>Ticket Category</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Ticket Updated Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -503,6 +508,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -540,6 +546,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -577,6 +584,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -597,7 +605,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -612,6 +620,11 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>Software</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-01-31 16:24:43</t>
         </is>
       </c>
     </row>
@@ -653,6 +666,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -692,6 +706,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -729,6 +744,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -768,6 +784,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -807,6 +824,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -844,6 +862,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -881,6 +900,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -920,6 +940,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -957,6 +978,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -994,6 +1016,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1033,6 +1056,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1070,6 +1094,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1109,6 +1134,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1146,6 +1172,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1185,6 +1212,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1222,6 +1250,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1259,6 +1288,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1298,6 +1328,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1337,6 +1368,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1374,6 +1406,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1411,6 +1444,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1448,6 +1482,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1487,6 +1522,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1524,6 +1560,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1561,6 +1598,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1598,6 +1636,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1637,6 +1676,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1676,6 +1716,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1713,6 +1754,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1750,6 +1792,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1787,6 +1830,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1826,6 +1870,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1863,6 +1908,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1902,6 +1948,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1939,6 +1986,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1976,6 +2024,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2015,6 +2064,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2052,6 +2102,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2089,6 +2140,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2126,6 +2178,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2165,6 +2218,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2204,6 +2258,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2241,6 +2296,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2278,6 +2334,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2317,6 +2374,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2354,6 +2412,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2393,6 +2452,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2432,6 +2492,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2471,6 +2532,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2508,6 +2570,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2545,6 +2608,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2584,6 +2648,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2623,6 +2688,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2662,6 +2728,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2699,6 +2766,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2736,6 +2804,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2773,6 +2842,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2810,6 +2880,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2847,6 +2918,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2884,6 +2956,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2921,6 +2994,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2960,6 +3034,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2999,6 +3074,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3009,7 +3085,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3034,6 +3110,11 @@
       <c r="I69" t="inlineStr">
         <is>
           <t>Hardware</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-01-31 16:18:51</t>
         </is>
       </c>
     </row>
@@ -3075,6 +3156,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3112,6 +3194,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3151,6 +3234,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3188,6 +3272,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3225,6 +3310,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3262,6 +3348,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3299,6 +3386,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3336,6 +3424,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3373,6 +3462,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3412,6 +3502,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3449,6 +3540,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3486,6 +3578,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3523,6 +3616,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3562,6 +3656,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3599,6 +3694,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3636,6 +3732,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3675,6 +3772,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3712,6 +3810,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3749,6 +3848,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3786,6 +3886,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3823,6 +3924,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3860,6 +3962,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3897,6 +4000,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3936,6 +4040,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3975,6 +4080,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4012,6 +4118,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4049,6 +4156,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4086,6 +4194,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4123,6 +4232,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4160,6 +4270,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4197,6 +4308,7 @@
           <t>Hardware</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4236,6 +4348,7 @@
           <t>Software</t>
         </is>
       </c>
+      <c r="J101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>